<commit_message>
update sta cell outlines
</commit_message>
<xml_diff>
--- a/STA Outlines/STA Cell Outline Names.xlsx
+++ b/STA Outlines/STA Cell Outline Names.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d612b085ce925e02/Desktop/SAV-Survey-Figures/STA Outlines/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\ad.sfwmd.gov\dfsroot\data\rsd_sta\STA_vegetation\STA_Vegetation_monitoring\SAV Surveys\R Script for Map and Figure Creation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{75F30413-A49D-49F3-AC71-A9D38237FDC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{977B43F3-12FA-4033-AD3D-4FB5C1AE37C9}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75F30413-A49D-49F3-AC71-A9D38237FDC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="58560" yWindow="960" windowWidth="21600" windowHeight="11235" xr2:uid="{48D7FE87-0ABA-4D31-B615-F0E9B6B19885}"/>
+    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{48D7FE87-0ABA-4D31-B615-F0E9B6B19885}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -306,13 +306,13 @@
     <t>STA-1W C8</t>
   </si>
   <si>
-    <t>STA1W_6_11</t>
-  </si>
-  <si>
-    <t>STA1W_7_11</t>
-  </si>
-  <si>
-    <t>STA1W_8_11</t>
+    <t>STA1W_8_24</t>
+  </si>
+  <si>
+    <t>STA1W_7_24</t>
+  </si>
+  <si>
+    <t>STA1W_6_24</t>
   </si>
 </sst>
 </file>
@@ -666,9 +666,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -706,7 +706,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -812,7 +812,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -954,7 +954,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1105,7 +1105,7 @@
         <v>87</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>88</v>
@@ -1127,7 +1127,7 @@
         <v>91</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>92</v>
@@ -1327,4 +1327,283 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E9778737509B994EB45D437017FC8FA0" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b7035606f42e21153edfad75bf939e77">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="66b9e29a-8983-41f2-b583-a83501d0124d" xmlns:ns3="a59002c2-3ea9-422d-b03a-3bc9df7a71c9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="20a6333f06af52356f18f51af80b5982" ns2:_="" ns3:_="">
+    <xsd:import namespace="66b9e29a-8983-41f2-b583-a83501d0124d"/>
+    <xsd:import namespace="a59002c2-3ea9-422d-b03a-3bc9df7a71c9"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="66b9e29a-8983-41f2-b583-a83501d0124d" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="MediaServiceAutoTags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="13" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="14" nillable="true" ma:displayName="MediaServiceLocation" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="18" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="20" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="12185140-ecae-4b08-a6d3-e60ccb92ce03" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="22" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="23" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="24" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="a59002c2-3ea9-422d-b03a-3bc9df7a71c9" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="11" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="12" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{ef2f3f46-251f-4b29-9527-9807fa135bb0}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="a59002c2-3ea9-422d-b03a-3bc9df7a71c9">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="66b9e29a-8983-41f2-b583-a83501d0124d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="a59002c2-3ea9-422d-b03a-3bc9df7a71c9" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2278F33C-7464-47FC-954F-E67402CD5C12}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0932C39B-2746-4701-A048-119E4349B4E8}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F67AF6A5-6934-40EF-A87A-C219A1C7EFD1}"/>
 </file>
</xml_diff>